<commit_message>
Swap columns: Service Level (A) now leads, Software Edition (B) follows
https://claude.ai/code/session_01CWL3KTXwhdHErbXSC2Xn3f
</commit_message>
<xml_diff>
--- a/Financial_Template.xlsx
+++ b/Financial_Template.xlsx
@@ -505,12 +505,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Service Level</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Software Edition</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Service Level</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -555,12 +555,12 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
+          <t>SaaS</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
           <t>Premium</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>SaaS</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -626,12 +626,12 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>SaaS</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>MPS</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -697,12 +697,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>SaaS</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>BPO</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -768,12 +768,12 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>MPS</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>SaaS</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -839,12 +839,12 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>MPS</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
           <t>Professional</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>MPS</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -910,12 +910,12 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>MPS</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>BPO</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -981,12 +981,12 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>BPO</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>SaaS</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -1052,12 +1052,12 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>BPO</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>MPS</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -1123,12 +1123,12 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
+          <t>BPO</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
           <t>Enterprise</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>BPO</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -1242,12 +1242,12 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
+          <t>SaaS</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
           <t>Premium</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>SaaS</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -1313,12 +1313,12 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>SaaS</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>MPS</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
@@ -1384,12 +1384,12 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>SaaS</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>BPO</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -1455,12 +1455,12 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>MPS</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>SaaS</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -1526,12 +1526,12 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
+          <t>MPS</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
           <t>Professional</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>MPS</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -1597,12 +1597,12 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Professional</t>
+          <t>MPS</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>BPO</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
@@ -1668,12 +1668,12 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>BPO</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>SaaS</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -1739,12 +1739,12 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>BPO</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>MPS</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
@@ -1810,12 +1810,12 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
+          <t>BPO</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
           <t>Enterprise</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>BPO</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">

</xml_diff>